<commit_message>
feat(kiet): complete remaining frontend pages, admin previews, QA suite, and sync project plan/report
</commit_message>
<xml_diff>
--- a/docs/plan_sheets/FoodFinder_Project_Plan.xlsx
+++ b/docs/plan_sheets/FoodFinder_Project_Plan.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,11 +108,17 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
+      <color rgb="00166534"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
       <color rgb="0092400E"/>
       <sz val="9.5"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -145,14 +151,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8FAFC"/>
         <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -242,10 +254,10 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -624,7 +636,7 @@
     <col width="65" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="47" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
@@ -705,7 +717,7 @@
       </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="8">
-        <f>COUNTIF('📋 Phân Công Task Chi Tiết'!G4:G24, "Done")</f>
+        <f>COUNTIF('📋 Phân Công Task Chi Tiết'!G4:G24, "Done")+COUNTIF('📋 Phân Công Task Chi Tiết'!G4:G24, "Completed")</f>
         <v/>
       </c>
       <c r="J5" s="4" t="n"/>
@@ -775,7 +787,7 @@
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Database", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")</f>
+        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Database", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")+COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Database", '📋 Phân Công Task Chi Tiết'!G4:G24, "Completed")</f>
         <v/>
       </c>
       <c r="E10" s="12">
@@ -805,7 +817,7 @@
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Backend", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")</f>
+        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Backend", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")+COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Backend", '📋 Phân Công Task Chi Tiết'!G4:G24, "Completed")</f>
         <v/>
       </c>
       <c r="E11" s="12">
@@ -835,7 +847,7 @@
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Frontend", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")</f>
+        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Frontend", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")+COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Frontend", '📋 Phân Công Task Chi Tiết'!G4:G24, "Completed")</f>
         <v/>
       </c>
       <c r="E12" s="12">
@@ -865,7 +877,7 @@
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Admin", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")</f>
+        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Admin", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")+COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Admin", '📋 Phân Công Task Chi Tiết'!G4:G24, "Completed")</f>
         <v/>
       </c>
       <c r="E13" s="12">
@@ -895,7 +907,7 @@
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "QA &amp; Testing", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")</f>
+        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "QA &amp; Testing", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")+COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "QA &amp; Testing", '📋 Phân Công Task Chi Tiết'!G4:G24, "Completed")</f>
         <v/>
       </c>
       <c r="E14" s="12">
@@ -925,7 +937,7 @@
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Documentation", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")</f>
+        <f>COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Documentation", '📋 Phân Công Task Chi Tiết'!G4:G24, "Done")+COUNTIFS('📋 Phân Công Task Chi Tiết'!B4:B24, "Documentation", '📋 Phân Công Task Chi Tiết'!G4:G24, "Completed")</f>
         <v/>
       </c>
       <c r="E15" s="12">
@@ -1136,7 +1148,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hướng dẫn: Cập nhật trạng thái (To Do, In Progress, In Review, Done) và Người phụ trách để Dashboard tự động tính toán</t>
+          <t>Hướng dẫn: Cập nhật trạng thái (To Do, In Progress, In Review, Done, Completed) và Người phụ trách để Dashboard tự động tính toán</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1242,7 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H4" s="12" t="inlineStr">
@@ -1245,7 +1257,7 @@
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K4" s="13" t="inlineStr">
@@ -1287,7 +1299,7 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H5" s="18" t="inlineStr">
@@ -1302,7 +1314,7 @@
       </c>
       <c r="J5" s="18" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K5" s="20" t="inlineStr">
@@ -1344,7 +1356,7 @@
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H6" s="12" t="inlineStr">
@@ -1359,7 +1371,7 @@
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K6" s="13" t="inlineStr">
@@ -1391,17 +1403,17 @@
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>Frontend Dev</t>
-        </is>
-      </c>
-      <c r="F7" s="17" t="inlineStr">
+          <t>Tuấn Kiệt</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="inlineStr">
         <is>
           <t>P2 - Trung bình</t>
         </is>
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H7" s="18" t="inlineStr">
@@ -1416,7 +1428,7 @@
       </c>
       <c r="J7" s="18" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K7" s="20" t="inlineStr">
@@ -1458,7 +1470,7 @@
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H8" s="12" t="inlineStr">
@@ -1473,7 +1485,7 @@
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
@@ -1515,7 +1527,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
@@ -1530,7 +1542,7 @@
       </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K9" s="20" t="inlineStr">
@@ -1572,7 +1584,7 @@
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
@@ -1587,7 +1599,7 @@
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">
@@ -1622,14 +1634,14 @@
           <t>Backend Dev</t>
         </is>
       </c>
-      <c r="F11" s="17" t="inlineStr">
+      <c r="F11" s="21" t="inlineStr">
         <is>
           <t>P2 - Trung bình</t>
         </is>
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
@@ -1644,7 +1656,7 @@
       </c>
       <c r="J11" s="18" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K11" s="20" t="inlineStr">
@@ -1676,7 +1688,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Frontend Dev</t>
+          <t>Tuấn Kiệt</t>
         </is>
       </c>
       <c r="F12" s="16" t="inlineStr">
@@ -1686,7 +1698,7 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
@@ -1701,7 +1713,7 @@
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K12" s="13" t="inlineStr">
@@ -1733,17 +1745,17 @@
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>Frontend Dev</t>
-        </is>
-      </c>
-      <c r="F13" s="17" t="inlineStr">
+          <t>Tuấn Kiệt</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="inlineStr">
         <is>
           <t>P2 - Trung bình</t>
         </is>
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H13" s="18" t="inlineStr">
@@ -1758,7 +1770,7 @@
       </c>
       <c r="J13" s="18" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K13" s="20" t="inlineStr">
@@ -1790,17 +1802,17 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Frontend Dev</t>
-        </is>
-      </c>
-      <c r="F14" s="17" t="inlineStr">
+          <t>Tuấn Kiệt</t>
+        </is>
+      </c>
+      <c r="F14" s="21" t="inlineStr">
         <is>
           <t>P2 - Trung bình</t>
         </is>
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H14" s="12" t="inlineStr">
@@ -1815,7 +1827,7 @@
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K14" s="13" t="inlineStr">
@@ -1855,7 +1867,7 @@
           <t>P1 - Cao</t>
         </is>
       </c>
-      <c r="G15" s="17" t="inlineStr">
+      <c r="G15" s="21" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
@@ -1912,7 +1924,7 @@
           <t>P1 - Cao</t>
         </is>
       </c>
-      <c r="G16" s="17" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
@@ -1969,7 +1981,7 @@
           <t>P1 - Cao</t>
         </is>
       </c>
-      <c r="G17" s="17" t="inlineStr">
+      <c r="G17" s="21" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
@@ -2026,7 +2038,7 @@
           <t>P3 - Thấp</t>
         </is>
       </c>
-      <c r="G18" s="17" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
@@ -2075,17 +2087,17 @@
       </c>
       <c r="E19" s="19" t="inlineStr">
         <is>
-          <t>Fullstack Dev</t>
-        </is>
-      </c>
-      <c r="F19" s="17" t="inlineStr">
+          <t>Tuấn Kiệt</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr">
         <is>
           <t>P2 - Trung bình</t>
         </is>
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H19" s="18" t="inlineStr">
@@ -2100,7 +2112,7 @@
       </c>
       <c r="J19" s="18" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K19" s="20" t="inlineStr">
@@ -2132,7 +2144,7 @@
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Fullstack Dev</t>
+          <t>Tuấn Kiệt</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -2142,7 +2154,7 @@
       </c>
       <c r="G20" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H20" s="12" t="inlineStr">
@@ -2157,7 +2169,7 @@
       </c>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K20" s="13" t="inlineStr">
@@ -2189,7 +2201,7 @@
       </c>
       <c r="E21" s="19" t="inlineStr">
         <is>
-          <t>Tester / QA</t>
+          <t>Tuấn Kiệt</t>
         </is>
       </c>
       <c r="F21" s="16" t="inlineStr">
@@ -2199,7 +2211,7 @@
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H21" s="18" t="inlineStr">
@@ -2214,7 +2226,7 @@
       </c>
       <c r="J21" s="18" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K21" s="20" t="inlineStr">
@@ -2246,17 +2258,17 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Tester / QA</t>
-        </is>
-      </c>
-      <c r="F22" s="17" t="inlineStr">
+          <t>Tuấn Kiệt</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
         <is>
           <t>P2 - Trung bình</t>
         </is>
       </c>
       <c r="G22" s="17" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="H22" s="12" t="inlineStr">
@@ -2271,7 +2283,7 @@
       </c>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="K22" s="13" t="inlineStr">
@@ -2306,12 +2318,12 @@
           <t>Team Leader</t>
         </is>
       </c>
-      <c r="F23" s="17" t="inlineStr">
+      <c r="F23" s="21" t="inlineStr">
         <is>
           <t>P2 - Trung bình</t>
         </is>
       </c>
-      <c r="G23" s="17" t="inlineStr">
+      <c r="G23" s="21" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
@@ -2363,12 +2375,12 @@
           <t>All Team</t>
         </is>
       </c>
-      <c r="F24" s="17" t="inlineStr">
+      <c r="F24" s="21" t="inlineStr">
         <is>
           <t>P2 - Trung bình</t>
         </is>
       </c>
-      <c r="G24" s="17" t="inlineStr">
+      <c r="G24" s="21" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
@@ -2397,7 +2409,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="G4:G24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"To Do,In Progress,In Review,Done"</formula1>
+      <formula1>"To Do,In Progress,In Review,Done,Completed"</formula1>
     </dataValidation>
     <dataValidation sqref="F4:F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P1 - Cao,P2 - Trung bình,P3 - Thấp"</formula1>
@@ -2421,10 +2433,10 @@
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="59" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2482,22 +2494,22 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Thành viên 1 (Điền tên)</t>
+          <t>52400207 - Phạm Nguyễn Tuấn Kiệt</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>Team Leader &amp; Fullstack</t>
+          <t>Frontend &amp; UI/UX Lead, Admin CMS, QA &amp; Testing</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Quản lý tiến độ, Kiến trúc hệ thống, Backend Lộ trình, Tài liệu đồ án</t>
+          <t>Mock Data (DB-04), Bộ lọc cấp 1 (FE-01), Marker &amp; Popup (FE-02), Card &amp; Chi tiết (FE-03), Admin CMS (ADM-01, ADM-02), Kiểm thử (QA-01, QA-02)</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>Phụ trách tổng</t>
+          <t>Hoàn thành 100% (8/8 tasks)</t>
         </is>
       </c>
     </row>
@@ -2507,22 +2519,22 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Thành viên 2 (Điền tên)</t>
+          <t>52400230 - Nguyễn Trọng Quý</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>Frontend Specialist</t>
+          <t>Database Architect, Data Engineering &amp; Docs</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Giao diện Lộ trình (Timeline, Modal), Bản đồ Leaflet Polyline, UX/UI</t>
+          <t>Thiết kế Schema mở rộng (DB-01), Danh mục 3 nhóm (DB-02), Seed 50+ địa điểm thực tế (DB-03), Báo cáo kỹ thuật &amp; ERD (DOC-01)</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Lead Frontend</t>
+          <t>Lead Database &amp; Docs</t>
         </is>
       </c>
     </row>
@@ -2532,50 +2544,26 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Thành viên 3 (Điền tên)</t>
+          <t>52400217 - Trần Hữu Nam</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>Backend &amp; Database</t>
+          <t>Backend API, Routing Algorithm &amp; Itinerary UI</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Database migration, API đề xuất lộ trình, Seed data Du lịch/Vui chơi</t>
+          <t>REST API Địa điểm &amp; Lộ trình (BE-01..BE-04), Giao diện Modal, Timeline, Leaflet Polyline &amp; Chia sẻ Lộ trình (FE-04..FE-07)</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>Lead Backend</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Thành viên 4 (Điền tên)</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>QA, Testing &amp; Data</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Kiểm thử thuật toán GPS, Thu thập 30+ địa điểm, Slide &amp; Demo đồ án</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>Lead QA &amp; Demo</t>
-        </is>
-      </c>
-    </row>
+          <t>Lead Backend &amp; Routing</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10"/>
     <row r="11"/>
     <row r="12">
@@ -2598,22 +2586,22 @@
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>Trọng Quý (DB/Docs)</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>Frontend Dev</t>
+          <t>Tuấn Kiệt (FE/Admin/QA)</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>Backend Dev</t>
+          <t>Hữu Nam (BE/Routing)</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>QA &amp; Data</t>
+          <t>Ghi Chú</t>
         </is>
       </c>
     </row>
@@ -2626,24 +2614,24 @@
           <t>Thiết kế Schema CSDL &amp; Thu thập dữ liệu Du lịch/Vui chơi</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E14" s="22" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F14" s="22" t="inlineStr">
-        <is>
-          <t>R</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>DB-01, DB-02, DB-03</t>
         </is>
       </c>
     </row>
@@ -2653,27 +2641,27 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>Xây dựng Thuật toán &amp; API Đề xuất Lộ trình</t>
-        </is>
-      </c>
-      <c r="C15" s="21" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
+          <t>Đồng bộ Mock Data Frontend 50 địa điểm &amp; 15 danh mục</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E15" s="22" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>DB-04</t>
         </is>
       </c>
     </row>
@@ -2683,27 +2671,27 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Thiết kế Giao diện Timeline &amp; Thiết lập lộ trình</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D16" s="22" t="inlineStr">
+          <t>Xây dựng Thuật toán &amp; API Đề xuất Lộ trình</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>BE-01, BE-02, BE-03, BE-04</t>
         </is>
       </c>
     </row>
@@ -2713,12 +2701,12 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Vẽ đường nối Leaflet Polyline &amp; Mở Google Maps</t>
-        </is>
-      </c>
-      <c r="C17" s="21" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>Nâng cấp bộ lọc đa dạng, Marker phân màu &amp; Card chi tiết</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
       <c r="D17" s="22" t="inlineStr">
@@ -2733,7 +2721,7 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>FE-01, FE-02, FE-03</t>
         </is>
       </c>
     </row>
@@ -2743,27 +2731,27 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Nâng cấp bộ lọc đa dạng (Ăn uống / Du lịch / Vui chơi)</t>
-        </is>
-      </c>
-      <c r="C18" s="21" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D18" s="22" t="inlineStr">
+          <t>Thiết kế Giao diện Timeline, Polyline &amp; Chia sẻ lộ trình</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>FE-04, FE-05, FE-06, FE-07</t>
         </is>
       </c>
     </row>
@@ -2773,27 +2761,27 @@
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Cập nhật Admin CMS &amp; Thống kê</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
+          <t>Cập nhật Admin CMS &amp; Thống kê Dashboard mở rộng</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E19" s="22" t="inlineStr">
+      <c r="D19" s="22" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>ADM-01, ADM-02</t>
         </is>
       </c>
     </row>
@@ -2806,24 +2794,24 @@
           <t>Kiểm thử Thuật toán GPS &amp; Responsive Mobile</t>
         </is>
       </c>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F20" s="22" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>QA-01, QA-02</t>
         </is>
       </c>
     </row>
@@ -2851,9 +2839,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="F21" s="22" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>DOC-01, DOC-02</t>
         </is>
       </c>
     </row>

</xml_diff>